<commit_message>
daily auto-refresh 2026-09-07 15:00
</commit_message>
<xml_diff>
--- a/daily_ethnicity_mix.xlsx
+++ b/daily_ethnicity_mix.xlsx
@@ -15657,16 +15657,16 @@
         <v>1</v>
       </c>
       <c r="K331" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="L331" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M331" t="n">
         <v>29</v>
       </c>
       <c r="N331" t="n">
-        <v>24</v>
+        <v>24.2</v>
       </c>
     </row>
     <row r="332">
@@ -35549,10 +35549,10 @@
         <v>0</v>
       </c>
       <c r="L436" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="M436" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="437">

</xml_diff>